<commit_message>
Update template for bill payment voucher.
</commit_message>
<xml_diff>
--- a/FinanceDataMigration/src/main/resources/migration-templates/BILL_PAYMENT_VOUCHER.xlsx
+++ b/FinanceDataMigration/src/main/resources/migration-templates/BILL_PAYMENT_VOUCHER.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <workbookPr/>
   <bookViews>
-    <workbookView xWindow="360" yWindow="15" windowWidth="20955" windowHeight="9720" activeTab="1"/>
+    <workbookView xWindow="360" yWindow="15" windowWidth="20955" windowHeight="9720" activeTab="0"/>
   </bookViews>
   <sheets>
     <sheet name="Bill Payment Voucher" sheetId="1" state="visible" r:id="rId2"/>
@@ -334,7 +334,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="63">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="62">
   <si>
     <t xml:space="preserve">BILL PAYMENT VOUCHER</t>
   </si>
@@ -345,7 +345,7 @@
     <t>S.No.</t>
   </si>
   <si>
-    <t xml:space="preserve">Voucher Group ID</t>
+    <t xml:space="preserve">Voucher Group Id</t>
   </si>
   <si>
     <t xml:space="preserve">ULB Name</t>
@@ -393,7 +393,7 @@
     <t>Gurugram</t>
   </si>
   <si>
-    <t>28/10/2026</t>
+    <t>31/10/2026</t>
   </si>
   <si>
     <t xml:space="preserve">Municipal Fund</t>
@@ -411,37 +411,37 @@
     <t xml:space="preserve">State Bank of India</t>
   </si>
   <si>
-    <t xml:space="preserve">Main Branch Panchkula</t>
-  </si>
-  <si>
-    <t>SBIN0001509</t>
-  </si>
-  <si>
-    <t>34767783281</t>
+    <t xml:space="preserve">India Gate</t>
+  </si>
+  <si>
+    <t>SBIN0000167</t>
+  </si>
+  <si>
+    <t>1234567890</t>
   </si>
   <si>
     <t xml:space="preserve">Cheque payments</t>
   </si>
   <si>
-    <t>DEPT_5/WBILL/0042/2026-27</t>
-  </si>
-  <si>
-    <t>DEPT_5/WBILL/0043/2026-27</t>
-  </si>
-  <si>
-    <t>DEPT_5/WBILL/0044/2026-27</t>
+    <t>DEPT_1/WBILL/0101/2026-27</t>
+  </si>
+  <si>
+    <t>DEPT_1/WBILL/0104/2026-27</t>
+  </si>
+  <si>
+    <t>DEPT_1/WBILL/0102/2026-27</t>
   </si>
   <si>
     <t>PV002</t>
   </si>
   <si>
-    <t>DEPT_5/WBILL/0050/2026-27</t>
+    <t>DEPT_1/WBILL/0106/2026-27</t>
   </si>
   <si>
     <t>PV003</t>
   </si>
   <si>
-    <t>DEPT_5/WBILL/0058/2026-27</t>
+    <t>DEPT_1/WBILL/0108/2026-27</t>
   </si>
   <si>
     <t xml:space="preserve">HOW TO FILL THE BILL PAYMENT VOUCHER TEMPLATE</t>
@@ -453,83 +453,80 @@
     <t xml:space="preserve">Enter a sequential S.No. for each Excel row.</t>
   </si>
   <si>
-    <t xml:space="preserve">2. Voucher Group Id</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Enter a voucher group id like PV001, PV002. If two or more than two voucher has group payment then mention same voucher group id same like PV001, PV001 and so on.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3. ULB Name</t>
+    <t xml:space="preserve">2. ULB Name</t>
   </si>
   <si>
     <t xml:space="preserve">Enter the name of the Urban Local Body for the row.</t>
   </si>
   <si>
-    <t xml:space="preserve">4. One row per bill</t>
+    <t xml:space="preserve">3. One row per bill</t>
   </si>
   <si>
     <t xml:space="preserve">Enter one row for each bill being paid.</t>
   </si>
   <si>
-    <t xml:space="preserve">5. Grouping bills</t>
+    <t xml:space="preserve">4. Grouping bills</t>
   </si>
   <si>
     <t xml:space="preserve">The API supports multiple bills in one payment voucher. Since Migration Reference has been removed, the reader needs an agreed grouping rule (for example, consecutive rows with identical voucher-level details) to combine bills into one request.</t>
   </si>
   <si>
-    <t xml:space="preserve">6. Voucher-level fields</t>
+    <t xml:space="preserve">5. Voucher-level fields</t>
   </si>
   <si>
     <t xml:space="preserve">Payment date, ULB, fund, function, department, payment mode, bank details, and description should be identical for rows belonging to the same voucher.</t>
   </si>
   <si>
-    <t xml:space="preserve">7. Required fields</t>
+    <t xml:space="preserve">6. Required fields</t>
   </si>
   <si>
     <t xml:space="preserve">All API fields are required except Description. Bill Number and Payment Amount are required for every bill row.</t>
   </si>
   <si>
-    <t xml:space="preserve">8. Date format</t>
+    <t xml:space="preserve">7. Date format</t>
   </si>
   <si>
     <t xml:space="preserve">Use dd/MM/yyyy, for example 27/10/2026.</t>
   </si>
   <si>
-    <t xml:space="preserve">9. Payment mode</t>
+    <t xml:space="preserve">8. Payment mode</t>
   </si>
   <si>
     <t xml:space="preserve">Only CHEQUE, NEFT, or RTGS are accepted by the API.</t>
   </si>
   <si>
-    <t xml:space="preserve">10. Payment amount</t>
+    <t xml:space="preserve">9. Payment amount</t>
   </si>
   <si>
     <t xml:space="preserve">Must be greater than 0 and have no more than two decimal places.</t>
   </si>
   <si>
-    <t xml:space="preserve">11. Finance master data</t>
+    <t xml:space="preserve">10. Finance master data</t>
   </si>
   <si>
     <t xml:space="preserve">Fund, function, department, bank, branch, and bank account must be valid in the target Finance tenant.</t>
   </si>
   <si>
-    <t xml:space="preserve">12. Existing bills</t>
+    <t xml:space="preserve">11. Existing bills</t>
   </si>
   <si>
     <t xml:space="preserve">Each Bill Number must identify a bill available in Finance and eligible for payment.</t>
   </si>
   <si>
-    <t xml:space="preserve">13. Sample data</t>
+    <t xml:space="preserve">12. Sample data</t>
   </si>
   <si>
     <t xml:space="preserve">Rows 5–7 on the first sheet are examples. Replace them with your actual migration data before uploading.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Important: This version treats each consecutive group with matching fields as one voucher. If two separate vouchers happen to have identical fields, put a blank row between them or add an explicit voucher reference column later. The current template has no unique voucher identifier.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="6">
+  <fonts count="7">
     <font>
       <sz val="11.000000"/>
       <color theme="1"/>
@@ -550,6 +547,10 @@
     <font>
       <b/>
       <color indexed="65"/>
+    </font>
+    <font>
+      <sz val="12.000000"/>
+      <name val="Times New Roman"/>
     </font>
     <font>
       <b/>
@@ -589,7 +590,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="4">
     <border>
       <left style="none"/>
       <right style="none"/>
@@ -612,11 +613,31 @@
       </bottom>
       <diagonal style="none"/>
     </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="thin">
+        <color rgb="FFD9E2F3"/>
+      </bottom>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="thin">
+        <color rgb="FFD9E2F3"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFD9E2F3"/>
+      </bottom>
+      <diagonal style="none"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="26">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
     <xf fontId="0" fillId="0" borderId="1" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -659,29 +680,36 @@
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf fontId="0" fillId="0" borderId="1" numFmtId="49" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf fontId="0" fillId="0" borderId="1" numFmtId="49" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf fontId="0" fillId="0" borderId="1" numFmtId="49" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf fontId="0" fillId="0" borderId="1" numFmtId="49" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf fontId="0" fillId="0" borderId="1" numFmtId="4" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf fontId="0" fillId="0" borderId="1" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf fontId="4" fillId="2" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf fontId="4" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf fontId="5" fillId="2" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf fontId="0" fillId="0" borderId="1" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0">
       <protection hidden="0" locked="1"/>
     </xf>
-    <xf fontId="5" fillId="3" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf fontId="0" fillId="5" borderId="1" numFmtId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf fontId="0" fillId="5" borderId="1" numFmtId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    <xf fontId="6" fillId="3" borderId="2" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf fontId="0" fillId="5" borderId="2" numFmtId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf fontId="6" fillId="3" borderId="3" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf fontId="0" fillId="5" borderId="3" numFmtId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -702,8 +730,8 @@
 
 <file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
 <personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <person displayName="OpenAI" id="{CFB4283E-B4DF-B889-ED3A-54B42DB697ED}"/>
-  <person displayName="OpenAI" id="{C028AC8C-8F94-A246-6A47-1C68E9A40664}"/>
+  <person displayName="OpenAI" id="{598B4DD1-42E9-EEFC-F91B-5C890BDCBD94}"/>
+  <person displayName="OpenAI" id="{CFA4ADD3-0BE7-6759-AC96-A157F819F6C1}"/>
 </personList>
 </file>
 
@@ -1187,59 +1215,59 @@
 
 <file path=xl/threadedComments/threadedComment1.xml><?xml version="1.0" encoding="utf-8"?>
 <ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <threadedComment ref="A4" personId="{CFB4283E-B4DF-B889-ED3A-54B42DB697ED}" id="{53F78006-5692-F4F1-FE41-4637D69FE9E6}" done="0">
+  <threadedComment ref="A4" personId="{598B4DD1-42E9-EEFC-F91B-5C890BDCBD94}" id="{53F78006-5692-F4F1-FE41-4637D69FE9E6}" done="0">
     <text xml:space="preserve">Serial number for the Excel row. Use sequential numbers.
 </text>
   </threadedComment>
-  <threadedComment ref="K4" personId="{C028AC8C-8F94-A246-6A47-1C68E9A40664}" id="{2DAC66FC-4AAA-67E8-D484-21C2E5136EB2}" done="0">
+  <threadedComment ref="K4" personId="{CFA4ADD3-0BE7-6759-AC96-A157F819F6C1}" id="{2DAC66FC-4AAA-67E8-D484-21C2E5136EB2}" done="0">
     <text xml:space="preserve">Required. IFSC code.
 </text>
   </threadedComment>
-  <threadedComment ref="L4" personId="{C028AC8C-8F94-A246-6A47-1C68E9A40664}" id="{7D67CAE5-CB8D-E679-A56B-D38C0CEBBE2B}" done="0">
+  <threadedComment ref="L4" personId="{CFA4ADD3-0BE7-6759-AC96-A157F819F6C1}" id="{7D67CAE5-CB8D-E679-A56B-D38C0CEBBE2B}" done="0">
     <text xml:space="preserve">Required. Bank account number must exist in Finance. Keep as text to preserve leading zeros.
 </text>
   </threadedComment>
-  <threadedComment ref="M4" personId="{C028AC8C-8F94-A246-6A47-1C68E9A40664}" id="{157037D5-36C6-154A-C92F-FC25DD9F0095}" done="0">
+  <threadedComment ref="M4" personId="{CFA4ADD3-0BE7-6759-AC96-A157F819F6C1}" id="{157037D5-36C6-154A-C92F-FC25DD9F0095}" done="0">
     <text xml:space="preserve">Optional. Maximum 1000 characters.
 </text>
   </threadedComment>
-  <threadedComment ref="N4" personId="{C028AC8C-8F94-A246-6A47-1C68E9A40664}" id="{0BDA7754-369D-FA0B-50E3-C4094CED978B}" done="0">
+  <threadedComment ref="N4" personId="{CFA4ADD3-0BE7-6759-AC96-A157F819F6C1}" id="{0BDA7754-369D-FA0B-50E3-C4094CED978B}" done="0">
     <text xml:space="preserve">Required. Existing bill number to be paid.
 </text>
   </threadedComment>
-  <threadedComment ref="O4" personId="{C028AC8C-8F94-A246-6A47-1C68E9A40664}" id="{60400F11-600F-995E-B8FD-853C67A798E8}" done="0">
+  <threadedComment ref="O4" personId="{CFA4ADD3-0BE7-6759-AC96-A157F819F6C1}" id="{60400F11-600F-995E-B8FD-853C67A798E8}" done="0">
     <text xml:space="preserve">Required. Amount to pay against this bill; greater than 0, maximum 2 decimal places.
 </text>
   </threadedComment>
-  <threadedComment ref="C4" personId="{C028AC8C-8F94-A246-6A47-1C68E9A40664}" id="{985D89D7-FFFD-20A3-29E5-D125261A5607}" done="0">
+  <threadedComment ref="C4" personId="{CFA4ADD3-0BE7-6759-AC96-A157F819F6C1}" id="{985D89D7-FFFD-20A3-29E5-D125261A5607}" done="0">
     <text xml:space="preserve">ULB name for this payment voucher.
 </text>
   </threadedComment>
-  <threadedComment ref="D4" personId="{C028AC8C-8F94-A246-6A47-1C68E9A40664}" id="{615BF305-EEEB-00AE-C6C8-113916FA4737}" done="0">
+  <threadedComment ref="D4" personId="{CFA4ADD3-0BE7-6759-AC96-A157F819F6C1}" id="{615BF305-EEEB-00AE-C6C8-113916FA4737}" done="0">
     <text xml:space="preserve">Required. Date format dd/MM/yyyy, e.g. 27/10/2026.
 </text>
   </threadedComment>
-  <threadedComment ref="E4" personId="{C028AC8C-8F94-A246-6A47-1C68E9A40664}" id="{59C5A379-3937-D446-5B71-ADDD8A9891C0}" done="0">
+  <threadedComment ref="E4" personId="{CFA4ADD3-0BE7-6759-AC96-A157F819F6C1}" id="{59C5A379-3937-D446-5B71-ADDD8A9891C0}" done="0">
     <text xml:space="preserve">Required. Fund name must match a fund configured in Finance.
 </text>
   </threadedComment>
-  <threadedComment ref="F4" personId="{C028AC8C-8F94-A246-6A47-1C68E9A40664}" id="{C47CC10D-D8F0-AF6E-50DD-201DADF92FA9}" done="0">
+  <threadedComment ref="F4" personId="{CFA4ADD3-0BE7-6759-AC96-A157F819F6C1}" id="{C47CC10D-D8F0-AF6E-50DD-201DADF92FA9}" done="0">
     <text xml:space="preserve">Required. Function name must match a function configured in Finance.
 </text>
   </threadedComment>
-  <threadedComment ref="G4" personId="{C028AC8C-8F94-A246-6A47-1C68E9A40664}" id="{E4A57EAC-3DED-B11D-F524-47736677247C}" done="0">
+  <threadedComment ref="G4" personId="{CFA4ADD3-0BE7-6759-AC96-A157F819F6C1}" id="{E4A57EAC-3DED-B11D-F524-47736677247C}" done="0">
     <text xml:space="preserve">Required. Department name must match the configured department.
 </text>
   </threadedComment>
-  <threadedComment ref="H4" personId="{C028AC8C-8F94-A246-6A47-1C68E9A40664}" id="{54D6D846-6EC2-5446-ADF8-B8EE041FEE66}" done="0">
+  <threadedComment ref="H4" personId="{CFA4ADD3-0BE7-6759-AC96-A157F819F6C1}" id="{54D6D846-6EC2-5446-ADF8-B8EE041FEE66}" done="0">
     <text xml:space="preserve">Required. Allowed values: CHEQUE, NEFT, RTGS.
 </text>
   </threadedComment>
-  <threadedComment ref="I4" personId="{C028AC8C-8F94-A246-6A47-1C68E9A40664}" id="{1346A7AA-CCEF-CE6D-D47C-5C95F0DF4CEB}" done="0">
+  <threadedComment ref="I4" personId="{CFA4ADD3-0BE7-6759-AC96-A157F819F6C1}" id="{1346A7AA-CCEF-CE6D-D47C-5C95F0DF4CEB}" done="0">
     <text xml:space="preserve">Required. Bank name must match the bank configuration.
 </text>
   </threadedComment>
-  <threadedComment ref="J4" personId="{C028AC8C-8F94-A246-6A47-1C68E9A40664}" id="{891C7670-DBB0-60D8-3550-3BC962FE591C}" done="0">
+  <threadedComment ref="J4" personId="{CFA4ADD3-0BE7-6759-AC96-A157F819F6C1}" id="{891C7670-DBB0-60D8-3550-3BC962FE591C}" done="0">
     <text xml:space="preserve">Required. Bank branch name.
 </text>
   </threadedComment>
@@ -1264,8 +1292,7 @@
     <col customWidth="1" min="13" max="13" style="1" width="28"/>
     <col customWidth="1" min="14" max="14" style="1" width="34"/>
     <col customWidth="1" min="15" max="15" style="1" width="18"/>
-    <col min="16" max="16" style="1" width="9.140625"/>
-    <col min="17" max="16384" style="1" width="9.140625"/>
+    <col min="16" max="16384" style="1" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1" ht="21">
@@ -1426,20 +1453,20 @@
         <v>29</v>
       </c>
       <c r="O5" s="12">
-        <v>220</v>
+        <v>7320</v>
       </c>
     </row>
     <row r="6" ht="14.25">
       <c r="A6" s="6">
         <v>2</v>
       </c>
-      <c r="B6" s="7" t="s">
+      <c r="B6" s="6" t="s">
         <v>17</v>
       </c>
       <c r="C6" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="D6" s="7" t="s">
+      <c r="D6" s="6" t="s">
         <v>19</v>
       </c>
       <c r="E6" s="8" t="s">
@@ -1454,16 +1481,16 @@
       <c r="H6" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="I6" s="9" t="s">
+      <c r="I6" s="8" t="s">
         <v>24</v>
       </c>
-      <c r="J6" s="9" t="s">
+      <c r="J6" s="8" t="s">
         <v>25</v>
       </c>
-      <c r="K6" s="10" t="s">
+      <c r="K6" s="13" t="s">
         <v>26</v>
       </c>
-      <c r="L6" s="10" t="s">
+      <c r="L6" s="13" t="s">
         <v>27</v>
       </c>
       <c r="M6" s="8" t="s">
@@ -1473,14 +1500,14 @@
         <v>30</v>
       </c>
       <c r="O6" s="12">
-        <v>751.65999999999997</v>
+        <v>75220</v>
       </c>
     </row>
     <row r="7" ht="14.25">
       <c r="A7" s="6">
         <v>3</v>
       </c>
-      <c r="B7" s="7" t="s">
+      <c r="B7" s="6" t="s">
         <v>17</v>
       </c>
       <c r="C7" s="8" t="s">
@@ -1501,16 +1528,16 @@
       <c r="H7" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="I7" s="9" t="s">
+      <c r="I7" s="8" t="s">
         <v>24</v>
       </c>
-      <c r="J7" s="9" t="s">
+      <c r="J7" s="8" t="s">
         <v>25</v>
       </c>
-      <c r="K7" s="10" t="s">
+      <c r="K7" s="13" t="s">
         <v>26</v>
       </c>
-      <c r="L7" s="10" t="s">
+      <c r="L7" s="13" t="s">
         <v>27</v>
       </c>
       <c r="M7" s="8" t="s">
@@ -1520,7 +1547,7 @@
         <v>31</v>
       </c>
       <c r="O7" s="12">
-        <v>123</v>
+        <v>23</v>
       </c>
     </row>
     <row r="8" ht="14.25">
@@ -1554,20 +1581,20 @@
       <c r="J8" s="8" t="s">
         <v>25</v>
       </c>
-      <c r="K8" s="13" t="s">
+      <c r="K8" s="14" t="s">
         <v>26</v>
       </c>
-      <c r="L8" s="13" t="s">
+      <c r="L8" s="14" t="s">
         <v>27</v>
       </c>
       <c r="M8" s="8" t="s">
         <v>28</v>
       </c>
-      <c r="N8" s="11" t="s">
+      <c r="N8" s="15" t="s">
         <v>33</v>
       </c>
       <c r="O8" s="12">
-        <v>1223</v>
+        <v>61220</v>
       </c>
     </row>
     <row r="9" ht="14.25">
@@ -1614,7 +1641,7 @@
         <v>35</v>
       </c>
       <c r="O9" s="12">
-        <v>1223</v>
+        <v>3220</v>
       </c>
     </row>
     <row r="10" ht="14.25">
@@ -1628,28 +1655,28 @@
       <c r="H10" s="1"/>
       <c r="I10" s="1"/>
       <c r="J10" s="1"/>
-      <c r="K10" s="14"/>
-      <c r="L10" s="14"/>
+      <c r="K10" s="1"/>
+      <c r="L10" s="1"/>
       <c r="M10" s="1"/>
-      <c r="N10" s="14"/>
-      <c r="O10" s="15"/>
+      <c r="N10" s="1"/>
+      <c r="O10" s="1"/>
     </row>
     <row r="11" ht="14.25">
-      <c r="A11" s="1"/>
-      <c r="B11" s="1"/>
-      <c r="C11" s="1"/>
-      <c r="D11" s="1"/>
-      <c r="E11" s="1"/>
-      <c r="F11" s="1"/>
-      <c r="G11" s="1"/>
-      <c r="H11" s="1"/>
-      <c r="I11" s="1"/>
-      <c r="J11" s="1"/>
-      <c r="K11" s="14"/>
-      <c r="L11" s="14"/>
-      <c r="M11" s="1"/>
-      <c r="N11" s="14"/>
-      <c r="O11" s="15"/>
+      <c r="A11" s="6"/>
+      <c r="B11" s="6"/>
+      <c r="C11" s="8"/>
+      <c r="D11" s="6"/>
+      <c r="E11" s="8"/>
+      <c r="F11" s="8"/>
+      <c r="G11" s="8"/>
+      <c r="H11" s="6"/>
+      <c r="I11" s="8"/>
+      <c r="J11" s="8"/>
+      <c r="K11" s="13"/>
+      <c r="L11" s="13"/>
+      <c r="M11" s="8"/>
+      <c r="N11" s="16"/>
+      <c r="O11" s="12"/>
     </row>
     <row r="12" ht="14.25">
       <c r="A12" s="1"/>
@@ -1662,11 +1689,11 @@
       <c r="H12" s="1"/>
       <c r="I12" s="1"/>
       <c r="J12" s="1"/>
-      <c r="K12" s="14"/>
-      <c r="L12" s="14"/>
+      <c r="K12" s="17"/>
+      <c r="L12" s="17"/>
       <c r="M12" s="1"/>
-      <c r="N12" s="14"/>
-      <c r="O12" s="15"/>
+      <c r="N12" s="17"/>
+      <c r="O12" s="18"/>
     </row>
     <row r="13" ht="14.25">
       <c r="A13" s="1"/>
@@ -1679,11 +1706,11 @@
       <c r="H13" s="1"/>
       <c r="I13" s="1"/>
       <c r="J13" s="1"/>
-      <c r="K13" s="14"/>
-      <c r="L13" s="14"/>
+      <c r="K13" s="17"/>
+      <c r="L13" s="17"/>
       <c r="M13" s="1"/>
-      <c r="N13" s="14"/>
-      <c r="O13" s="15"/>
+      <c r="N13" s="17"/>
+      <c r="O13" s="18"/>
     </row>
     <row r="14" ht="14.25">
       <c r="A14" s="1"/>
@@ -1696,11 +1723,11 @@
       <c r="H14" s="1"/>
       <c r="I14" s="1"/>
       <c r="J14" s="1"/>
-      <c r="K14" s="14"/>
-      <c r="L14" s="14"/>
+      <c r="K14" s="17"/>
+      <c r="L14" s="17"/>
       <c r="M14" s="1"/>
-      <c r="N14" s="14"/>
-      <c r="O14" s="15"/>
+      <c r="N14" s="17"/>
+      <c r="O14" s="18"/>
     </row>
     <row r="15" ht="14.25">
       <c r="A15" s="1"/>
@@ -1713,11 +1740,11 @@
       <c r="H15" s="1"/>
       <c r="I15" s="1"/>
       <c r="J15" s="1"/>
-      <c r="K15" s="14"/>
-      <c r="L15" s="14"/>
+      <c r="K15" s="17"/>
+      <c r="L15" s="17"/>
       <c r="M15" s="1"/>
-      <c r="N15" s="14"/>
-      <c r="O15" s="15"/>
+      <c r="N15" s="17"/>
+      <c r="O15" s="18"/>
     </row>
     <row r="16" ht="14.25">
       <c r="A16" s="1"/>
@@ -1730,11 +1757,11 @@
       <c r="H16" s="1"/>
       <c r="I16" s="1"/>
       <c r="J16" s="1"/>
-      <c r="K16" s="14"/>
-      <c r="L16" s="14"/>
+      <c r="K16" s="17"/>
+      <c r="L16" s="17"/>
       <c r="M16" s="1"/>
-      <c r="N16" s="14"/>
-      <c r="O16" s="15"/>
+      <c r="N16" s="17"/>
+      <c r="O16" s="18"/>
     </row>
     <row r="17" ht="14.25">
       <c r="A17" s="1"/>
@@ -1747,11 +1774,11 @@
       <c r="H17" s="1"/>
       <c r="I17" s="1"/>
       <c r="J17" s="1"/>
-      <c r="K17" s="14"/>
-      <c r="L17" s="14"/>
+      <c r="K17" s="17"/>
+      <c r="L17" s="17"/>
       <c r="M17" s="1"/>
-      <c r="N17" s="14"/>
-      <c r="O17" s="15"/>
+      <c r="N17" s="17"/>
+      <c r="O17" s="18"/>
     </row>
     <row r="18" ht="14.25">
       <c r="A18" s="1"/>
@@ -1764,11 +1791,11 @@
       <c r="H18" s="1"/>
       <c r="I18" s="1"/>
       <c r="J18" s="1"/>
-      <c r="K18" s="14"/>
-      <c r="L18" s="14"/>
+      <c r="K18" s="17"/>
+      <c r="L18" s="17"/>
       <c r="M18" s="1"/>
-      <c r="N18" s="14"/>
-      <c r="O18" s="15"/>
+      <c r="N18" s="17"/>
+      <c r="O18" s="18"/>
     </row>
     <row r="19" ht="14.25">
       <c r="A19" s="1"/>
@@ -1781,11 +1808,11 @@
       <c r="H19" s="1"/>
       <c r="I19" s="1"/>
       <c r="J19" s="1"/>
-      <c r="K19" s="14"/>
-      <c r="L19" s="14"/>
+      <c r="K19" s="17"/>
+      <c r="L19" s="17"/>
       <c r="M19" s="1"/>
-      <c r="N19" s="14"/>
-      <c r="O19" s="15"/>
+      <c r="N19" s="17"/>
+      <c r="O19" s="18"/>
     </row>
     <row r="20" ht="14.25">
       <c r="A20" s="1"/>
@@ -1798,11 +1825,11 @@
       <c r="H20" s="1"/>
       <c r="I20" s="1"/>
       <c r="J20" s="1"/>
-      <c r="K20" s="14"/>
-      <c r="L20" s="14"/>
+      <c r="K20" s="17"/>
+      <c r="L20" s="17"/>
       <c r="M20" s="1"/>
-      <c r="N20" s="14"/>
-      <c r="O20" s="15"/>
+      <c r="N20" s="17"/>
+      <c r="O20" s="18"/>
     </row>
     <row r="21" ht="14.25">
       <c r="A21" s="1"/>
@@ -1815,11 +1842,11 @@
       <c r="H21" s="1"/>
       <c r="I21" s="1"/>
       <c r="J21" s="1"/>
-      <c r="K21" s="14"/>
-      <c r="L21" s="14"/>
+      <c r="K21" s="17"/>
+      <c r="L21" s="17"/>
       <c r="M21" s="1"/>
-      <c r="N21" s="14"/>
-      <c r="O21" s="15"/>
+      <c r="N21" s="17"/>
+      <c r="O21" s="18"/>
     </row>
     <row r="22" ht="14.25">
       <c r="A22" s="1"/>
@@ -1832,11 +1859,11 @@
       <c r="H22" s="1"/>
       <c r="I22" s="1"/>
       <c r="J22" s="1"/>
-      <c r="K22" s="14"/>
-      <c r="L22" s="14"/>
+      <c r="K22" s="17"/>
+      <c r="L22" s="17"/>
       <c r="M22" s="1"/>
-      <c r="N22" s="14"/>
-      <c r="O22" s="15"/>
+      <c r="N22" s="17"/>
+      <c r="O22" s="18"/>
     </row>
     <row r="23" ht="14.25">
       <c r="A23" s="1"/>
@@ -1849,11 +1876,11 @@
       <c r="H23" s="1"/>
       <c r="I23" s="1"/>
       <c r="J23" s="1"/>
-      <c r="K23" s="14"/>
-      <c r="L23" s="14"/>
+      <c r="K23" s="17"/>
+      <c r="L23" s="17"/>
       <c r="M23" s="1"/>
-      <c r="N23" s="14"/>
-      <c r="O23" s="15"/>
+      <c r="N23" s="17"/>
+      <c r="O23" s="18"/>
     </row>
     <row r="24" ht="14.25">
       <c r="A24" s="1"/>
@@ -1866,11 +1893,11 @@
       <c r="H24" s="1"/>
       <c r="I24" s="1"/>
       <c r="J24" s="1"/>
-      <c r="K24" s="14"/>
-      <c r="L24" s="14"/>
+      <c r="K24" s="17"/>
+      <c r="L24" s="17"/>
       <c r="M24" s="1"/>
-      <c r="N24" s="14"/>
-      <c r="O24" s="15"/>
+      <c r="N24" s="17"/>
+      <c r="O24" s="18"/>
     </row>
     <row r="25" ht="14.25">
       <c r="A25" s="1"/>
@@ -1883,11 +1910,45 @@
       <c r="H25" s="1"/>
       <c r="I25" s="1"/>
       <c r="J25" s="1"/>
-      <c r="K25" s="14"/>
-      <c r="L25" s="14"/>
+      <c r="K25" s="17"/>
+      <c r="L25" s="17"/>
       <c r="M25" s="1"/>
-      <c r="N25" s="14"/>
-      <c r="O25" s="15"/>
+      <c r="N25" s="17"/>
+      <c r="O25" s="18"/>
+    </row>
+    <row r="26" ht="14.25">
+      <c r="A26" s="1"/>
+      <c r="B26" s="1"/>
+      <c r="C26" s="1"/>
+      <c r="D26" s="1"/>
+      <c r="E26" s="1"/>
+      <c r="F26" s="1"/>
+      <c r="G26" s="1"/>
+      <c r="H26" s="1"/>
+      <c r="I26" s="1"/>
+      <c r="J26" s="1"/>
+      <c r="K26" s="17"/>
+      <c r="L26" s="17"/>
+      <c r="M26" s="1"/>
+      <c r="N26" s="17"/>
+      <c r="O26" s="18"/>
+    </row>
+    <row r="27" ht="14.25">
+      <c r="A27" s="1"/>
+      <c r="B27" s="1"/>
+      <c r="C27" s="1"/>
+      <c r="D27" s="1"/>
+      <c r="E27" s="1"/>
+      <c r="F27" s="1"/>
+      <c r="G27" s="1"/>
+      <c r="H27" s="1"/>
+      <c r="I27" s="1"/>
+      <c r="J27" s="1"/>
+      <c r="K27" s="17"/>
+      <c r="L27" s="17"/>
+      <c r="M27" s="1"/>
+      <c r="N27" s="17"/>
+      <c r="O27" s="18"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -1901,38 +1962,74 @@
   <legacyDrawing r:id="rId3"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
-      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="6" disablePrompts="0">
-        <x14:dataValidation xr:uid="{4B770CC9-C0CE-4B4E-8ED4-7CC6C269FB6D}" type="list" allowBlank="0" error="Select CHEQUE, NEFT, or RTGS." errorStyle="stop" errorTitle="Invalid payment mode" imeMode="noControl" operator="between" showDropDown="0" showErrorMessage="0" showInputMessage="0">
+      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="12" disablePrompts="0">
+        <x14:dataValidation xr:uid="{73AAD0F7-A751-4161-B688-F1AE356BBBAD}" type="list" allowBlank="0" error="Select CHEQUE, NEFT, or RTGS." errorStyle="stop" errorTitle="Invalid payment mode" imeMode="noControl" operator="between" showDropDown="0" showErrorMessage="0" showInputMessage="0">
           <x14:formula1>
             <xm:f>"CHEQUE,NEFT,RTGS"</xm:f>
           </x14:formula1>
-          <xm:sqref>H5:H6 H10:H25 H7</xm:sqref>
+          <xm:sqref>H5 H12:H27</xm:sqref>
         </x14:dataValidation>
-        <x14:dataValidation xr:uid="{A5F3C778-3B45-4FC5-BFDA-7783ED397553}" type="decimal" allowBlank="0" error="Payment amount must be greater than zero." errorStyle="stop" errorTitle="Invalid payment amount" imeMode="noControl" operator="greaterThan" showDropDown="0" showErrorMessage="0" showInputMessage="0">
+        <x14:dataValidation xr:uid="{205AB112-D76C-45F5-9A0B-0F2D03888A83}" type="decimal" allowBlank="0" error="Payment amount must be greater than zero." errorStyle="stop" errorTitle="Invalid payment amount" imeMode="noControl" operator="greaterThan" showDropDown="0" showErrorMessage="0" showInputMessage="0">
           <x14:formula1>
             <xm:f>0</xm:f>
           </x14:formula1>
-          <xm:sqref>O5:O7 O10:O25</xm:sqref>
+          <xm:sqref>O5 O12:O27</xm:sqref>
         </x14:dataValidation>
-        <x14:dataValidation xr:uid="{4D07ED0D-4C8C-4050-9FAB-FABFD0B09528}" type="list" allowBlank="0" error="Select CHEQUE, NEFT, or RTGS." errorStyle="stop" errorTitle="Invalid payment mode" imeMode="noControl" operator="between" showDropDown="0" showErrorMessage="0" showInputMessage="0">
+        <x14:dataValidation xr:uid="{46F89B32-9D35-436F-9ACD-B14BDB07DE1E}" type="list" allowBlank="0" error="Select CHEQUE, NEFT, or RTGS." errorStyle="stop" errorTitle="Invalid payment mode" imeMode="noControl" operator="between" showDropDown="0" showErrorMessage="0" showInputMessage="0">
+          <x14:formula1>
+            <xm:f>"CHEQUE,NEFT,RTGS"</xm:f>
+          </x14:formula1>
+          <xm:sqref>H11</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation xr:uid="{729CAE25-5CD5-4C6F-9F86-5E613593CCF0}" type="decimal" allowBlank="0" error="Payment amount must be greater than zero." errorStyle="stop" errorTitle="Invalid payment amount" imeMode="noControl" operator="greaterThan" showDropDown="0" showErrorMessage="0" showInputMessage="0">
+          <x14:formula1>
+            <xm:f>0</xm:f>
+          </x14:formula1>
+          <xm:sqref>O11</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation xr:uid="{72B9D740-1ADE-4F5C-9D35-E96C62EDF4ED}" type="list" allowBlank="0" error="Select CHEQUE, NEFT, or RTGS." errorStyle="stop" errorTitle="Invalid payment mode" imeMode="noControl" operator="between" showDropDown="0" showErrorMessage="0" showInputMessage="0">
+          <x14:formula1>
+            <xm:f>"CHEQUE,NEFT,RTGS"</xm:f>
+          </x14:formula1>
+          <xm:sqref>H6</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation xr:uid="{71947D70-7226-4822-80DF-F3D32ACEDA08}" type="decimal" allowBlank="0" error="Payment amount must be greater than zero." errorStyle="stop" errorTitle="Invalid payment amount" imeMode="noControl" operator="greaterThan" showDropDown="0" showErrorMessage="0" showInputMessage="0">
+          <x14:formula1>
+            <xm:f>0</xm:f>
+          </x14:formula1>
+          <xm:sqref>O6</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation xr:uid="{41877DEC-18FF-42DD-BA5C-863BBDBBCE89}" type="list" allowBlank="0" error="Select CHEQUE, NEFT, or RTGS." errorStyle="stop" errorTitle="Invalid payment mode" imeMode="noControl" operator="between" showDropDown="0" showErrorMessage="0" showInputMessage="0">
+          <x14:formula1>
+            <xm:f>"CHEQUE,NEFT,RTGS"</xm:f>
+          </x14:formula1>
+          <xm:sqref>H7</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation xr:uid="{75DBAFAB-A30F-4067-AF08-445074A73D68}" type="decimal" allowBlank="0" error="Payment amount must be greater than zero." errorStyle="stop" errorTitle="Invalid payment amount" imeMode="noControl" operator="greaterThan" showDropDown="0" showErrorMessage="0" showInputMessage="0">
+          <x14:formula1>
+            <xm:f>0</xm:f>
+          </x14:formula1>
+          <xm:sqref>O7</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation xr:uid="{575A3194-51AD-4B8F-89B6-8C8289B65163}" type="list" allowBlank="0" error="Select CHEQUE, NEFT, or RTGS." errorStyle="stop" errorTitle="Invalid payment mode" imeMode="noControl" operator="between" showDropDown="0" showErrorMessage="0" showInputMessage="0">
           <x14:formula1>
             <xm:f>"CHEQUE,NEFT,RTGS"</xm:f>
           </x14:formula1>
           <xm:sqref>H8</xm:sqref>
         </x14:dataValidation>
-        <x14:dataValidation xr:uid="{A3B6D30F-4988-484F-9922-EC661FB96B8C}" type="decimal" allowBlank="0" error="Payment amount must be greater than zero." errorStyle="stop" errorTitle="Invalid payment amount" imeMode="noControl" operator="greaterThan" showDropDown="0" showErrorMessage="0" showInputMessage="0">
+        <x14:dataValidation xr:uid="{17C072BE-7F3D-4963-859C-99E9D756A4A6}" type="decimal" allowBlank="0" error="Payment amount must be greater than zero." errorStyle="stop" errorTitle="Invalid payment amount" imeMode="noControl" operator="greaterThan" showDropDown="0" showErrorMessage="0" showInputMessage="0">
           <x14:formula1>
             <xm:f>0</xm:f>
           </x14:formula1>
           <xm:sqref>O8</xm:sqref>
         </x14:dataValidation>
-        <x14:dataValidation xr:uid="{F4666220-75F9-48FA-93C8-DC71345196FC}" type="list" allowBlank="0" error="Select CHEQUE, NEFT, or RTGS." errorStyle="stop" errorTitle="Invalid payment mode" imeMode="noControl" operator="between" showDropDown="0" showErrorMessage="0" showInputMessage="0">
+        <x14:dataValidation xr:uid="{1AB1FADF-494F-4AB5-AB46-57F997CBA0D4}" type="list" allowBlank="0" error="Select CHEQUE, NEFT, or RTGS." errorStyle="stop" errorTitle="Invalid payment mode" imeMode="noControl" operator="between" showDropDown="0" showErrorMessage="0" showInputMessage="0">
           <x14:formula1>
             <xm:f>"CHEQUE,NEFT,RTGS"</xm:f>
           </x14:formula1>
           <xm:sqref>H9</xm:sqref>
         </x14:dataValidation>
-        <x14:dataValidation xr:uid="{BB51DBFE-A4EF-4E68-8489-1D245BF32A27}" type="decimal" allowBlank="0" error="Payment amount must be greater than zero." errorStyle="stop" errorTitle="Invalid payment amount" imeMode="noControl" operator="greaterThan" showDropDown="0" showErrorMessage="0" showInputMessage="0">
+        <x14:dataValidation xr:uid="{3C3ED434-0334-4682-9FC3-EA0E4573C596}" type="decimal" allowBlank="0" error="Payment amount must be greater than zero." errorStyle="stop" errorTitle="Invalid payment amount" imeMode="noControl" operator="greaterThan" showDropDown="0" showErrorMessage="0" showInputMessage="0">
           <x14:formula1>
             <xm:f>0</xm:f>
           </x14:formula1>
@@ -1948,142 +2045,127 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col customWidth="1" min="1" max="1" style="16" width="23.140625"/>
-    <col customWidth="1" min="2" max="2" style="16" width="55.421875"/>
-    <col min="3" max="3" style="16" width="9.140625"/>
-    <col min="4" max="16384" style="16" width="9.140625"/>
+    <col customWidth="1" min="1" max="1" width="23.140625"/>
+    <col customWidth="1" min="2" max="2" width="55.421875"/>
   </cols>
   <sheetData>
-    <row r="1" ht="20.25">
-      <c r="A1" s="17" t="s">
+    <row r="1" ht="15">
+      <c r="A1" s="19"/>
+    </row>
+    <row r="3" ht="20.25">
+      <c r="A3" s="20" t="s">
         <v>36</v>
       </c>
-      <c r="B1" s="17"/>
-    </row>
-    <row r="2">
-      <c r="A2" s="18"/>
-      <c r="B2" s="18"/>
-    </row>
-    <row r="3" ht="14">
-      <c r="A3" s="19" t="s">
+      <c r="B3" s="20"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="21"/>
+      <c r="B4" s="21"/>
+    </row>
+    <row r="5" ht="14">
+      <c r="A5" s="22" t="s">
         <v>37</v>
       </c>
-      <c r="B3" s="20" t="s">
+      <c r="B5" s="23" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="4" ht="42.75">
-      <c r="A4" s="19" t="s">
+    <row r="6" ht="14">
+      <c r="A6" s="24" t="s">
         <v>39</v>
       </c>
-      <c r="B4" s="21" t="s">
+      <c r="B6" s="25" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="5" ht="14">
-      <c r="A5" s="19" t="s">
+    <row r="7" ht="14">
+      <c r="A7" s="24" t="s">
         <v>41</v>
       </c>
-      <c r="B5" s="20" t="s">
+      <c r="B7" s="25" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="6" ht="14">
-      <c r="A6" s="19" t="s">
+    <row r="8" ht="57">
+      <c r="A8" s="24" t="s">
         <v>43</v>
       </c>
-      <c r="B6" s="20" t="s">
+      <c r="B8" s="25" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="7" ht="57">
-      <c r="A7" s="19" t="s">
+    <row r="9" ht="42.75">
+      <c r="A9" s="24" t="s">
         <v>45</v>
       </c>
-      <c r="B7" s="20" t="s">
+      <c r="B9" s="25" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="8" ht="42.75">
-      <c r="A8" s="19" t="s">
+    <row r="10" ht="28.5">
+      <c r="A10" s="24" t="s">
         <v>47</v>
       </c>
-      <c r="B8" s="20" t="s">
+      <c r="B10" s="25" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="9" ht="28.5">
-      <c r="A9" s="19" t="s">
+    <row r="11" ht="14">
+      <c r="A11" s="24" t="s">
         <v>49</v>
       </c>
-      <c r="B9" s="20" t="s">
+      <c r="B11" s="25" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="10" ht="14">
-      <c r="A10" s="19" t="s">
+    <row r="12" ht="14">
+      <c r="A12" s="24" t="s">
         <v>51</v>
       </c>
-      <c r="B10" s="20" t="s">
+      <c r="B12" s="25" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="11" ht="14">
-      <c r="A11" s="19" t="s">
+    <row r="13" ht="28.5">
+      <c r="A13" s="24" t="s">
         <v>53</v>
       </c>
-      <c r="B11" s="20" t="s">
+      <c r="B13" s="25" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="12" ht="28.5">
-      <c r="A12" s="19" t="s">
+    <row r="14" ht="28.5">
+      <c r="A14" s="24" t="s">
         <v>55</v>
       </c>
-      <c r="B12" s="20" t="s">
+      <c r="B14" s="25" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="13" ht="28.5">
-      <c r="A13" s="19" t="s">
+    <row r="15" ht="28.5">
+      <c r="A15" s="24" t="s">
         <v>57</v>
       </c>
-      <c r="B13" s="20" t="s">
+      <c r="B15" s="25" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="14" ht="28.5">
-      <c r="A14" s="19" t="s">
+    <row r="16" ht="28.5">
+      <c r="A16" s="24" t="s">
         <v>59</v>
       </c>
-      <c r="B14" s="20" t="s">
+      <c r="B16" s="25" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="15" ht="28.5">
-      <c r="A15" s="19" t="s">
+    <row r="18" ht="19.5" customHeight="1">
+      <c r="A18" t="s">
         <v>61</v>
       </c>
-      <c r="B15" s="20" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="16"/>
-      <c r="B16" s="16"/>
-    </row>
-    <row r="17" ht="19.5" customHeight="1">
-      <c r="A17" s="16"/>
-    </row>
-    <row r="18">
-      <c r="A18" s="16"/>
-    </row>
-    <row r="19">
-      <c r="A19" s="16"/>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:B1"/>
+    <mergeCell ref="A3:B3"/>
   </mergeCells>
   <printOptions headings="0" gridLines="0"/>
   <pageMargins left="0.70078740157480324" right="0.70078740157480324" top="0.75196850393700787" bottom="0.75196850393700787" header="0.29999999999999999" footer="0.29999999999999999"/>

</xml_diff>